<commit_message>
fix: unify approval logic and align test cases
</commit_message>
<xml_diff>
--- a/docs/Casos_de_Pruebas_Funcionario.xlsx
+++ b/docs/Casos_de_Pruebas_Funcionario.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B7:K24"/>
+  <dimension ref="A7:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.25" customWidth="1" min="1" max="1"/>
@@ -513,40 +513,40 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>CP_RF02_01</t>
+          <t>CP_RF05_01</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Login exitoso como Funcionario
+          <t xml:space="preserve">Registrar revisión SAG como aprobada
 </t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sesión no iniciada. Sistema desplegado y accesible.</t>
+          <t>Sesión iniciada. Trámite TR-001-2026 en estado "en revisión".</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Usuario: carlos.munoz / Contraseña: 123456</t>
+          <t>Acción: marcar control SAG = Aprobado</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1- Abrir prototipo (prototipo.html).
-2- Presionar "Ingresar como Funcionario".
-3- Verificar que redirige al Panel de Control.</t>
+          <t>1- Seleccionar trámite TR-001-2026 en el dashboard.
+2- En sección "Controles SAG/PDI" hacer clic en "SAG: Aprobado".
+3- Guardar cambio.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra el Panel de Control con nombre "Carlos Muñoz – Funcionario SNA" y lista de trámites.</t>
+          <t>El estado del control SAG cambia a "Aprobado". La acción queda registrada en el historial con timestamp y nombre del funcionario.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Ruta = dashboard.</t>
+          <t>Control SAG = aprobado. Historial actualizado.</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
@@ -568,40 +568,40 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>CP_RF02_02</t>
+          <t>CP_RF08_01</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acceso bloqueado con campos vacíos
+          <t xml:space="preserve">Buscar trámite con código QR válido
 </t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Sesión no iniciada. Sistema desplegado.</t>
+          <t>Sesión iniciada. Trámite TR-002-2026 existe en el sistema.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Campos usuario y contraseña vacíos.</t>
+          <t>Código QR ingresado: "TR-002-2026"</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1- Abrir el prototipo.
-2- Dejar todos los campos en blanco.
-3- Presionar "Ingresar".</t>
+          <t>1- Ir a sección "Escanear QR".
+2- Ingresar "TR-002-2026" en el campo de texto.
+3- Presionar "Buscar Trámite".</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra mensaje de error indicando que los campos son requeridos. No permite el acceso.</t>
+          <t>El sistema muestra el detalle del trámite TR-002-2026 con datos del viajero, declaración SAG y estado actual.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Sesión no iniciada. Permanece en pantalla de login.</t>
+          <t>Vista de detalle del trámite TR-002-2026 activa.</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
@@ -623,40 +623,40 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>CP_RF05_01</t>
+          <t>CP_RF08_02</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar revisión SAG como aprobada
+          <t xml:space="preserve">Buscar trámite con código QR inválido
 </t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Trámite TR-001-2026 en estado "en revisión".</t>
+          <t>Sesión iniciada.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Acción: marcar control SAG = Aprobado</t>
+          <t>Código QR ingresado: "TR-999-XXXX" (no existe en el sistema).</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1- Seleccionar trámite TR-001-2026 en el dashboard.
-2- En sección "Controles SAG/PDI" hacer clic en "SAG: Aprobado".
-3- Guardar cambio.</t>
+          <t>1- Ir a "Escanear QR".
+2- Ingresar "TR-999-XXXX".
+3- Presionar "Buscar Trámite".</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>El estado del control SAG cambia a "Aprobado". La acción queda registrada en el historial con timestamp y nombre del funcionario.</t>
+          <t>El sistema muestra el mensaje: "No se encontró un trámite con ese código QR". No navega a ningún detalle.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Control SAG = aprobado. Historial actualizado.</t>
+          <t>Permanece en "Escanear QR". Sin trámite seleccionado.</t>
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr">
@@ -678,41 +678,40 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>CP_RF05_02</t>
+          <t>CP_RF08_03</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar revisión PDI como observado
+          <t xml:space="preserve">Buscar trámite con campo QR vacío
 </t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Trámite TR-003-2026 en estado "en revisión".</t>
+          <t>Sesión iniciada.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Acción: marcar control PDI = Observado; texto: "Documento con fecha próxima a vencer".</t>
+          <t>Campo QR: vacío.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>1- Seleccionar trámite TR-003-2026.
-2- En controles PDI, seleccionar "Observado".
-3- Ingresar texto de observación.
-4- Guardar.</t>
+          <t>1- Ir a "Escanear QR".
+2- Dejar el campo vacío.
+3- Presionar "Buscar Trámite" o tecla Enter.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Control PDI queda como "Observado". La observación queda registrada en historial con autor y timestamp.</t>
+          <t>El sistema muestra el mensaje "Ingrese un código QR válido" y no realiza búsqueda.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Control PDI = observado con nota. Historial actualizado.</t>
+          <t>Permanece en "Escanear QR". Ningún trámite seleccionado.</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
@@ -722,7 +721,7 @@
       </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
     </row>
@@ -734,40 +733,40 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>CP_RF05_03</t>
+          <t>CP_RF08_04</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intentar guardar control SAG sin seleccionar estado
+          <t xml:space="preserve">Buscar trámite presionando tecla Enter
 </t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Trámite TR-002-2026 en estado "en revisión".</t>
+          <t>Sesión iniciada. Trámite TR-004-2026 existe.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Ningún estado seleccionado para control SAG.</t>
+          <t>Código QR: "TR-004-2026"; acción: tecla Enter.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>1- Seleccionar trámite TR-002-2026.
-2- No seleccionar estado SAG.
-3- Presionar "Guardar".</t>
+          <t>1- Ir a "Escanear QR".
+2- Ingresar "TR-004-2026".
+3- Presionar tecla Enter.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra mensaje de validación: se debe seleccionar un estado para el control SAG. No guarda ningún cambio.</t>
+          <t>El sistema navega al detalle del trámite TR-004-2026, igual que al usar el botón "Buscar Trámite".</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>No se guarda ningún cambio. Trámite permanece con estado SAG vacío.</t>
+          <t>Vista de detalle del trámite TR-004-2026 activa.</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
@@ -789,40 +788,40 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>CP_RF08_01</t>
+          <t>CP_RF09_01</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buscar trámite con código QR válido
+          <t xml:space="preserve">Aprobar un trámite en estado "en revisión"
 </t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Trámite TR-002-2026 existe en el sistema.</t>
+          <t>Sesión iniciada. Trámite TR-001-2026 en estado "en revisión".</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Código QR ingresado: "TR-002-2026"</t>
+          <t>Acción: Aprobar trámite TR-001-2026.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1- Ir a sección "Escanear QR".
-2- Ingresar "TR-002-2026" en el campo de texto.
-3- Presionar "Buscar Trámite".</t>
+          <t>1- Buscar trámite TR-001-2026 (QR o dashboard).
+2- Presionar "Aprobar Trámite".
+3- Confirmar acción.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra el detalle del trámite TR-002-2026 con datos del viajero, declaración SAG y estado actual.</t>
+          <t>El estado cambia a "Aprobado". El historial registra las entradas de control SAG aprobado y control PDI aprobado, con timestamp y nombre del funcionario.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Vista de detalle del trámite TR-002-2026 activa.</t>
+          <t>Estado = aprobado. Controles SAG y PDI = aprobado. Historial actualizado.</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
@@ -844,40 +843,40 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>CP_RF08_02</t>
+          <t>CP_RF09_02</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buscar trámite con código QR inválido
+          <t xml:space="preserve">Rechazar un trámite en estado "en revisión"
 </t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada.</t>
+          <t>Sesión iniciada. Trámite TR-003-2026 en estado "en revisión".</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Código QR ingresado: "TR-999-XXXX" (no existe en el sistema).</t>
+          <t>Acción: Rechazar trámite TR-003-2026.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>1- Ir a "Escanear QR".
-2- Ingresar "TR-999-XXXX".
-3- Presionar "Buscar Trámite".</t>
+          <t>1- Buscar trámite TR-003-2026.
+2- Presionar "Rechazar Trámite".
+3- Confirmar acción.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra el mensaje: "No se encontró un trámite con ese código QR". No navega a ningún detalle.</t>
+          <t>El estado cambia a "Rechazado". El historial registra: fecha, acción y nombre del funcionario.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Permanece en "Escanear QR". Sin trámite seleccionado.</t>
+          <t>Estado = rechazado. Historial actualizado.</t>
         </is>
       </c>
       <c r="J15" s="1" t="inlineStr">
@@ -899,40 +898,40 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>CP_RF08_03</t>
+          <t>CP_RF09_03</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buscar trámite con campo QR vacío
+          <t xml:space="preserve">Aprobar un trámite ya aprobado
 </t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada.</t>
+          <t>Sesión iniciada. Trámite TR-004-2026 en estado "aprobado" con controles SAG y PDI aprobados.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Campo QR: vacío.</t>
+          <t>Acción: presionar "Aprobar Trámite" nuevamente.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1- Ir a "Escanear QR".
-2- Dejar el campo vacío.
-3- Presionar "Buscar Trámite" o tecla Enter.</t>
+          <t>1- Navegar al trámite TR-004-2026 (ya aprobado).
+2- Presionar "Aprobar Trámite".
+3- Revisar estado e historial.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra el mensaje "Ingrese un código QR válido" y no realiza búsqueda.</t>
+          <t>El estado permanece "Aprobado". Los controles SAG y PDI se mantienen en "Aprobado". El historial registra las nuevas entradas de control con timestamp.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Permanece en "Escanear QR". Ningún trámite seleccionado.</t>
+          <t>Estado = aprobado. Sin cambio de estado. Historial con nuevas entradas de control.</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">
@@ -942,7 +941,7 @@
       </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
     </row>
@@ -954,40 +953,40 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>CP_RF08_04</t>
+          <t>CP_RF10_02</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buscar trámite presionando tecla Enter
+          <t xml:space="preserve">Historial completo de cambios de estado
 </t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Sesión iniciada. Trámite TR-004-2026 existe.</t>
+          <t>Sesión iniciada. Trámite TR-001-2026 ha pasado por: pendiente → en revisión → aprobado.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Código QR: "TR-004-2026"; acción: tecla Enter.</t>
+          <t>Sin entradas adicionales; solo consulta del historial.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1- Ir a "Escanear QR".
-2- Ingresar "TR-004-2026".
-3- Presionar tecla Enter.</t>
+          <t>1- Navegar al trámite TR-001-2026.
+2- Desplazarse hasta la sección "Historial".
+3- Revisar cada entrada.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>El sistema navega al detalle del trámite TR-004-2026, igual que al usar el botón "Buscar Trámite".</t>
+          <t>El historial muestra al menos 3 entradas: (1) Creado/pendiente, (2) En revisión, (3) Aprobado — cada una con fecha ISO y nombre del funcionario.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Vista de detalle del trámite TR-004-2026 activa.</t>
+          <t>Historial visible e íntegro, sin entradas perdidas.</t>
         </is>
       </c>
       <c r="J17" s="1" t="inlineStr">
@@ -997,7 +996,7 @@
       </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
     </row>
@@ -1009,375 +1008,48 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>CP_RF09_01</t>
+          <t>CP_RF10_03</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aprobar un trámite en estado "en revisión"
-</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Trámite TR-001-2026 en estado "en revisión".</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Acción: Aprobar trámite TR-001-2026.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>1- Buscar trámite TR-001-2026 (QR o dashboard).
-2- Presionar "Aprobar Trámite".
-3- Confirmar acción.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>El estado cambia a "Aprobado". El historial registra: fecha, "Trámite aprobado", nombre del funcionario.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Estado = aprobado. Botones Aprobar/Rechazar deshabilitados.</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF09_02</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rechazar un trámite en estado "en revisión"
-</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Trámite TR-003-2026 en estado "en revisión".</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Acción: Rechazar trámite TR-003-2026.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>1- Buscar trámite TR-003-2026.
-2- Presionar "Rechazar Trámite".
-3- Confirmar acción.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>El estado cambia a "Rechazado". El historial registra: fecha, acción y nombre del funcionario.</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Estado = rechazado. Historial actualizado.</t>
-        </is>
-      </c>
-      <c r="J19" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K19" s="1" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF09_03</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intentar aprobar un trámite ya finalizado
-</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Trámite TR-005-2026 en estado "aprobado".</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Acción: intentar presionar "Aprobar Trámite".</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>1- Navegar al trámite TR-005-2026.
-2- Verificar estado del botón "Aprobar Trámite".</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>El botón "Aprobar Trámite" está visualmente deshabilitado. No es posible ejecutar la acción.</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Estado del trámite permanece "aprobado". Sin cambios en historial.</t>
-        </is>
-      </c>
-      <c r="J20" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K20" s="1" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF09_04</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aprobar trámite con menor sin autorización
-</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Existe trámite con menor de edad sin autorización de tutor cargada.</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Trámite con campo menor = true y sin documento de autorización de tutor.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>1- Abrir detalle del trámite con menor.
-2- Intentar presionar "Aprobar Trámite".</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>El sistema muestra advertencia: el trámite contiene un menor sin autorización válida. No aprueba automáticamente.</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Trámite no aprobado. El funcionario debe revisar la advertencia.</t>
-        </is>
-      </c>
-      <c r="J21" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K21" s="1" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF10_01</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estado cambia a "en revisión" al abrir trámite pendiente
-</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Trámite TR-004-2026 en estado "pendiente".</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Acción: seleccionar trámite TR-004-2026 desde el dashboard.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>1- En el dashboard, hacer clic sobre trámite TR-004-2026 (estado "pendiente").
-2- Observar el estado en la vista de detalle.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>El estado cambia de "pendiente" a "en revisión". El historial registra la apertura con fecha.</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Estado = en revisión. Historial contiene entrada de apertura.</t>
-        </is>
-      </c>
-      <c r="J22" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K22" s="1" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF10_02</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Historial completo de cambios de estado
-</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Sesión iniciada. Trámite TR-001-2026 ha pasado por: pendiente → en revisión → aprobado.</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Sin entradas adicionales; solo consulta del historial.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>1- Navegar al trámite TR-001-2026.
-2- Desplazarse hasta la sección "Historial".
-3- Revisar cada entrada.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>El historial muestra al menos 3 entradas: (1) Creado/pendiente, (2) En revisión, (3) Aprobado — cada una con fecha ISO y nombre del funcionario.</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Historial visible e íntegro, sin entradas perdidas.</t>
-        </is>
-      </c>
-      <c r="J23" s="1" t="inlineStr">
-        <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="K23" s="1" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>CP_RF10_03</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Estado no se revierte al volver al dashboard
 </t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Sesión iniciada. Trámite TR-002-2026 fue aprobado en la misma sesión.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Sin entradas adicionales.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1- Aprobar trámite TR-002-2026.
 2- Volver al dashboard.
 3- Reabrir trámite TR-002-2026.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>El trámite TR-002-2026 sigue mostrando estado "aprobado". El historial conserva el registro de aprobación.</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Estado persistido dentro de la sesión. Historial íntegro.</t>
         </is>
       </c>
-      <c r="J24" s="1" t="inlineStr">
+      <c r="J18" s="1" t="inlineStr">
         <is>
           <t>Abierto</t>
         </is>
       </c>
-      <c r="K24" s="1" t="inlineStr">
+      <c r="K18" s="1" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>

</xml_diff>